<commit_message>
Log this session's decisions in the QNL assumption log (QNL-023..028)
Record the manufacturer-metadata work and the Dar Cairo naming alignment as
assumption-log entries:

- QNL-023 metadata added in the reference-model row shapes, component sub-entities
- QNL-024 values/units taken from the Dar Cairo columns, not HQ's (HQ units wrong)
- QNL-025 metadata joins by index/mapping (HEX PHX->HEX, pumps, generator)
- QNL-026 FCU metadata via Euroclima selection-sheet expansion (94 units)
- QNL-027 FCU 2F 06-33 and the unmatchable families left without metadata
- QNL-028 Dar Cairo identifier alignment: datapoints to dashed English, equipment
  codes kept, rooms dashed, join keys preserved

Formatting reapplied with format_assumption_log.py.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01L1CU23wNWRi3FVm37EG2eh
</commit_message>
<xml_diff>
--- a/projects/Assumption_Log.xlsx
+++ b/projects/Assumption_Log.xlsx
@@ -49,7 +49,7 @@
       <color rgb="FF808080"/>
     </font>
   </fonts>
-  <fills count="13">
+  <fills count="15">
     <fill>
       <patternFill/>
     </fill>
@@ -111,6 +111,16 @@
         <fgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DEEAF6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -153,7 +163,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -199,6 +209,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -744,7 +760,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.21875" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -1508,6 +1524,276 @@
         <is>
           <t>6</t>
         </is>
+      </c>
+    </row>
+    <row r="17" ht="58.05" customHeight="1">
+      <c r="A17" s="11" t="inlineStr">
+        <is>
+          <t>QNL-023</t>
+        </is>
+      </c>
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="C17" s="17" t="inlineStr">
+        <is>
+          <t>Structure</t>
+        </is>
+      </c>
+      <c r="D17" s="11" t="inlineStr">
+        <is>
+          <t>Metadata</t>
+        </is>
+      </c>
+      <c r="E17" s="11" t="inlineStr">
+        <is>
+          <t>12 equipment families (AHU, FCU, DX, HEX, pumps, CCU, EF, generator, pressurisation, climate)</t>
+        </is>
+      </c>
+      <c r="F17" s="11" t="inlineStr">
+        <is>
+          <t>Manufacturer datasheets give properties per component (cooling coil, fans, motors, outdoor unit)</t>
+        </is>
+      </c>
+      <c r="G17" s="11" t="inlineStr">
+        <is>
+          <t>Added the 16 metadata predicates in the Dar Cairo/SSC/HQ row shapes: literals as props, quantities as &lt;blanknode&gt; value+unit; component properties on brick:hasPart sub-entities (CHW-Coil, SF, RF, Motor, OD) - all Brick 1.4 classes, no para: minted</t>
+        </is>
+      </c>
+      <c r="H17" s="11" t="inlineStr">
+        <is>
+          <t>The three reference models attach component metadata to sub-entities and write quantities as blanknodes</t>
+        </is>
+      </c>
+      <c r="I17" s="11" t="n">
+        <v>977</v>
+      </c>
+    </row>
+    <row r="18" ht="58.05" customHeight="1">
+      <c r="A18" s="11" t="inlineStr">
+        <is>
+          <t>QNL-024</t>
+        </is>
+      </c>
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="C18" s="13" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="D18" s="11" t="inlineStr">
+        <is>
+          <t>Metadata</t>
+        </is>
+      </c>
+      <c r="E18" s="11" t="inlineStr">
+        <is>
+          <t>All quantity metadata rows</t>
+        </is>
+      </c>
+      <c r="F18" s="11" t="inlineStr">
+        <is>
+          <t>QF HQ v0.4 carries several wrong brick:hasUnit (air flow as unit:V, cooling capacity as unit:HZ)</t>
+        </is>
+      </c>
+      <c r="G18" s="11" t="inlineStr">
+        <is>
+          <t>Took brick:value and brick:hasUnit from the workbook's 'Value (Dar Cairo)' / 'Unit (QUDT)' columns, never HQ's</t>
+        </is>
+      </c>
+      <c r="H18" s="11" t="inlineStr">
+        <is>
+          <t>Dar Cairo is the unit authority; HQ's own README documents its units as wrong</t>
+        </is>
+      </c>
+      <c r="I18" s="11" t="n">
+        <v>882</v>
+      </c>
+    </row>
+    <row r="19" ht="58.05" customHeight="1">
+      <c r="A19" s="11" t="inlineStr">
+        <is>
+          <t>QNL-025</t>
+        </is>
+      </c>
+      <c r="B19" s="11" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="C19" s="18" t="inlineStr">
+        <is>
+          <t>Identifier</t>
+        </is>
+      </c>
+      <c r="D19" s="11" t="inlineStr">
+        <is>
+          <t>Metadata</t>
+        </is>
+      </c>
+      <c r="E19" s="11" t="inlineStr">
+        <is>
+          <t>Heat exchangers, pumps, generator</t>
+        </is>
+      </c>
+      <c r="F19" s="11" t="inlineStr">
+        <is>
+          <t>Datasheets tag them PHX/B/01-05, CHWP/B/01-04, 'GENERATOR SET'; the ontology has HEX01-05, CHW_P01-04, ELEC_Gen</t>
+        </is>
+      </c>
+      <c r="G19" s="11" t="inlineStr">
+        <is>
+          <t>Joined HEX by index (PHX/B/0n -&gt; HEX0n, user-confirmed), pumps CHWP/B/0n -&gt; CHW_P0n, generator -&gt; ELEC_Gen</t>
+        </is>
+      </c>
+      <c r="H19" s="11" t="inlineStr">
+        <is>
+          <t>Prefixes differ but the units correspond 1:1 by number/position</t>
+        </is>
+      </c>
+      <c r="I19" s="11" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="20" ht="58.05" customHeight="1">
+      <c r="A20" s="11" t="inlineStr">
+        <is>
+          <t>QNL-026</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="C20" s="16" t="inlineStr">
+        <is>
+          <t>Scope</t>
+        </is>
+      </c>
+      <c r="D20" s="11" t="inlineStr">
+        <is>
+          <t>Metadata</t>
+        </is>
+      </c>
+      <c r="E20" s="11" t="inlineStr">
+        <is>
+          <t>FCU family - 94 of 137 units</t>
+        </is>
+      </c>
+      <c r="F20" s="11" t="inlineStr">
+        <is>
+          <t>FCU datasheets are 28 Euroclima selection sheets keyed by position (B/03,04; 1F/04-54), one model per group</t>
+        </is>
+      </c>
+      <c r="G20" s="11" t="inlineStr">
+        <is>
+          <t>Expanded each selection-sheet tag to the FCUs it names and wrote its model/capacity/flow/power to every unit in the group</t>
+        </is>
+      </c>
+      <c r="H20" s="11" t="inlineStr">
+        <is>
+          <t>The selection sheet groups identical units under one model; the group tag names them explicitly</t>
+        </is>
+      </c>
+      <c r="I20" s="11" t="n">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="21" ht="58.05" customHeight="1">
+      <c r="A21" s="11" t="inlineStr">
+        <is>
+          <t>QNL-027</t>
+        </is>
+      </c>
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="C21" s="16" t="inlineStr">
+        <is>
+          <t>Scope</t>
+        </is>
+      </c>
+      <c r="D21" s="11" t="inlineStr">
+        <is>
+          <t>Metadata</t>
+        </is>
+      </c>
+      <c r="E21" s="11" t="inlineStr">
+        <is>
+          <t>FCU 2F 06-33; closed control units; climate &amp; pressurisation units; out-of-range CAV/VAV/EF</t>
+        </is>
+      </c>
+      <c r="F21" s="11" t="inlineStr">
+        <is>
+          <t>Their datasheet tags do not correspond to any ontology entity (2F numbers 06-33 vs 034-062; CC/B vs CCU_808n; no MCG/PU entity; units absent from the register)</t>
+        </is>
+      </c>
+      <c r="G21" s="11" t="inlineStr">
+        <is>
+          <t>Left them without metadata and reported every tag in QNL_metadata_join_report.csv; did not guess a join</t>
+        </is>
+      </c>
+      <c r="H21" s="11" t="inlineStr">
+        <is>
+          <t>User confirmed FCU 2F 06-33 are different units, not a numbering offset; the rest have no matching entity - do not assume metadata a source cannot place</t>
+        </is>
+      </c>
+      <c r="I21" s="11" t="n">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="22" ht="58.05" customHeight="1">
+      <c r="A22" s="11" t="inlineStr">
+        <is>
+          <t>QNL-028</t>
+        </is>
+      </c>
+      <c r="B22" s="11" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="C22" s="18" t="inlineStr">
+        <is>
+          <t>Identifier</t>
+        </is>
+      </c>
+      <c r="D22" s="11" t="inlineStr">
+        <is>
+          <t>All layers</t>
+        </is>
+      </c>
+      <c r="E22" s="11" t="inlineStr">
+        <is>
+          <t>Every subject/object identifier</t>
+        </is>
+      </c>
+      <c r="F22" s="11" t="inlineStr">
+        <is>
+          <t>Points were named as BMS tokens (AvgSpcHumd_PV, RunSts); equipment/rooms used '_' between word-parts</t>
+        </is>
+      </c>
+      <c r="G22" s="11" t="inlineStr">
+        <is>
+          <t>Aligned to Dar Cairo: datapoints renamed to dashed English from label or class (Return-Temperature, Run-Status); equipment/part tags kept their industry codes (AHU, SF, CHW-Coil) with '_'-&gt;'-' within the tag; 277 room name-words dashed. ref:hasTimeseriesId/para:hasEntityId untouched; crosswalk written</t>
+        </is>
+      </c>
+      <c r="H22" s="11" t="inlineStr">
+        <is>
+          <t>Client asked to match Dar Cairo's naming convention; camelCase 71%-&gt;0%, join keys preserved via the crosswalk</t>
+        </is>
+      </c>
+      <c r="I22" s="11" t="n">
+        <v>3753</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Hold CHWPU-P02 at the building until its floor is confirmed on site
The only basis for putting it in the basement was that its pair CHWPU-P01 sits
in B-220_Plant-Room-04 - inference from a sibling, not a source, and the one of
the four retargets that no document supported. The other three stand: two on
tag level tokens verified against 337 located assets, one on an explicit Level
statement in the metadata workbook.

Twenty-four assets now sit at the building, three on a floor.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01G5ei61eJmqXtuLmQFDtSnt
</commit_message>
<xml_diff>
--- a/projects/Assumption_Log.xlsx
+++ b/projects/Assumption_Log.xlsx
@@ -2520,7 +2520,7 @@
       </c>
       <c r="E38" s="11" t="inlineStr">
         <is>
-          <t>4 assets retargeted from the building to a floor</t>
+          <t>3 assets retargeted from the building to a floor</t>
         </is>
       </c>
       <c r="F38" s="11" t="inlineStr">
@@ -2530,17 +2530,17 @@
       </c>
       <c r="G38" s="11" t="inlineStr">
         <is>
-          <t>entity:QNL_CAV-1F-S15-001 -&gt; entity:QNL_L1; entity:QNL_VAV-B-S13-005 -&gt; entity:QNL_B; entity:QNL_DX-RP21 -&gt; entity:QNL_P; entity:QNL_CHWPU-P02 -&gt; entity:QNL_B.</t>
+          <t>entity:QNL_CAV-1F-S15-001 -&gt; entity:QNL_L1; entity:QNL_VAV-B-S13-005 -&gt; entity:QNL_B; entity:QNL_DX-RP21 -&gt; entity:QNL_P. entity:QNL_CHWPU-P02 was considered and deliberately LEFT at the building.</t>
         </is>
       </c>
       <c r="H38" s="11" t="inlineStr">
         <is>
-          <t>Evidence per asset. CAV-1F-S15-001: the 1F tag token, which resolves to Level 1 on 134 of the 135 located assets that carry it. VAV-B-S13-005: the B token, 202 of 202. DX-RP21: QNL_Full_Metadata.xlsx states Level "Roof level" and room served "PLC 8 / IDF ROOF PLANT"; entity:QNL_P is labelled "Roof Plant". CHWPU-P02 is the weakest of the four and is INFERRED, not sourced: its pair CHWPU-P01 is in entity:QNL_B-220_Plant-Room-04, and a duty/standby pump pair shares a plant room. Confirm on site.</t>
+          <t>Evidence per asset, and only where a source states it. CAV-1F-S15-001: the 1F tag token, which resolves to Level 1 on 134 of the 135 located assets that carry it. VAV-B-S13-005: the B token, 202 of 202. DX-RP21: QNL_Full_Metadata.xlsx states Level "Roof level" and room served "PLC 8 / IDF ROOF PLANT"; entity:QNL_P is labelled "Roof Plant". CHWPU-P02 was NOT moved: the only basis was that its pair CHWPU-P01 sits in entity:QNL_B-220_Plant-Room-04, which is inference from a sibling rather than a source. Client decision 2026-09-03 - hold it at the building until the floor is confirmed on site.</t>
         </is>
       </c>
       <c r="I38" s="11" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix assumption log: close QNL-047, add QNL-048
The previous commit pushed the ontology and handover note but the
assumption-log write failed with a tuple-instead-of-string cell value,
leaving the log stale relative to the other two.

- QNL-047 marked RESOLVED: all 50 per-fan TEF points added, no new
  classes needed. Records that FTSP/FTST were explained by the
  historian's own Description column.
- QNL-048 added: 1,314 historian tags of the same seven suffixes are
  unmodelled across 28 other equipment families. Left out deliberately
  as a scope call for the client, not by oversight.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01G5ei61eJmqXtuLmQFDtSnt
</commit_message>
<xml_diff>
--- a/projects/Assumption_Log.xlsx
+++ b/projects/Assumption_Log.xlsx
@@ -163,7 +163,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -215,6 +215,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -760,7 +763,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I41"/>
+  <dimension ref="A1:I42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.21875" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -2671,17 +2674,64 @@
       </c>
       <c r="G41" s="11" t="inlineStr">
         <is>
-          <t>Not added. Recorded as a scope question.</t>
+          <t>RESOLVED. All 50 added, with no new classes needed: FTSP -&gt; para:Fail_Stop_Alarm, FTST -&gt; para:Fail_Start_Alarm, FltRst -&gt; brick:Fault_Reset_Command, RuntimeMtr -&gt; brick:On_Timer_Sensor (unit:HR), StartsCtr -&gt; para:Start_Count, TripCtr -&gt; para:Trip_Count, RemSts -&gt; para:Remote_Status. All 131 historian TEF tags now resolve.</t>
         </is>
       </c>
       <c r="H41" s="11" t="inlineStr">
         <is>
-          <t>OPEN. These are per-FAN points, a different set from the 36 group points that were asked for and added. Under the skill's own rule an IO row with no point is a scope call, not a defect - the client decides whether the model needs them. Note FTSP and FTST are unexplained abbreviations; they want decoding before any class is chosen.</t>
+          <t>Client direction 2026-09-03. The two "unexplained" abbreviations were explained by the historian's own Description column, which had not been read closely enough: FTSP is "Fail to Stop Alarm" and FTST is "Fail to Start Alarm", both of which SSC had already coined para: classes for. The remaining five resolved on the ladder without coining anything new. These sit on the individual fans rather than the set, because the historian scopes them per fan: a runtime meter or starts counter is the evidence for duty/standby changeover, so averaging it at set level would destroy the one thing it is for.</t>
         </is>
       </c>
       <c r="I41" s="11" t="inlineStr">
         <is>
-          <t>0 (50 pending)</t>
+          <t>50 points, 200 rows</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="19" t="inlineStr">
+        <is>
+          <t>QNL-048</t>
+        </is>
+      </c>
+      <c r="B42" s="19" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="C42" s="19" t="inlineStr">
+        <is>
+          <t>Scope</t>
+        </is>
+      </c>
+      <c r="D42" s="19" t="inlineStr">
+        <is>
+          <t>Points</t>
+        </is>
+      </c>
+      <c r="E42" s="19" t="inlineStr">
+        <is>
+          <t>1,314 historian tags across 28 other equipment families</t>
+        </is>
+      </c>
+      <c r="F42" s="19" t="inlineStr">
+        <is>
+          <t>The cross-check that closed QNL-047 was run against the whole historian, not just the TEFs. The same seven suffixes (FTSP, FTST, FltRst, RuntimeMtr, StartsCtr, TripCtr, RemSts) appear on 28 other equipment families and are not modelled: VAV 247, AHU 146, ELE 145, FCU 137, EF 136, DX 120, CCU 62, SEF 62, CAV 51, SurfaceWtr 45, CHW 29, KEF 28, and the rest in ones and twos.</t>
+        </is>
+      </c>
+      <c r="G42" s="19" t="inlineStr">
+        <is>
+          <t>Not added. Recorded as a scope question for the client.</t>
+        </is>
+      </c>
+      <c r="H42" s="19" t="inlineStr">
+        <is>
+          <t>OPEN, and the largest remaining gap in the sheet - 1,314 points, roughly 2,628 rows, against the 19,546 the sheet holds today. Every class is already settled by QNL-046 and QNL-047, so adding them is mechanical rather than a modelling exercise. It is left out deliberately, not by oversight: the skill treats an IO row with no point as a scope call for the client, and adding 2,628 rows on our own initiative would be a material widening of what was asked for.</t>
+        </is>
+      </c>
+      <c r="I42" s="19" t="inlineStr">
+        <is>
+          <t>0 (1,314 pending)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Restore the 3 VAV-1F-S15-039S points
Client confirmed the selected list omits this box by oversight rather than
by decision: the asset register lists it in its own right serving L1-048
Staff Office, a room no other box serves, and the near-identical 039 is
selected. Leaving it out would have left that room with no VAV telemetry.

prune_to_selected.py now exempts the three tags by name alongside
ContributionFraction, each with its reason, so a re-run does not strip
them again. The sheet carries four unselected timeseries ids, all exempt
for stated reasons.

Sheet: 19,244 -> 19,250 rows, 10 errors unchanged, all tests pass.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01G5ei61eJmqXtuLmQFDtSnt
</commit_message>
<xml_diff>
--- a/projects/Assumption_Log.xlsx
+++ b/projects/Assumption_Log.xlsx
@@ -2778,7 +2778,7 @@
       </c>
       <c r="I43" s="19" t="inlineStr">
         <is>
-          <t>149 points, 302 rows</t>
+          <t>146 points, 296 rows net (149 removed, 3 restored under QNL-050)</t>
         </is>
       </c>
     </row>
@@ -2815,17 +2815,17 @@
       </c>
       <c r="G44" s="19" t="inlineStr">
         <is>
-          <t>Dropped the 3 points under QNL-049. The equipment entity is kept, with its location, feeds, isFedBy and IFC reference intact.</t>
+          <t>Dropped the 3 points under QNL-049, then RESTORED them on client confirmation the same day. The equipment entity was kept intact throughout. prune_to_selected.py now exempts the three tags by name, so a re-run does not strip them again.</t>
         </is>
       </c>
       <c r="H44" s="19" t="inlineStr">
         <is>
-          <t>OPEN - flagged for the client rather than resolved. This looks like an omission in the selection, not a decision: the box is real, it serves a room no other box serves, and the near-identical 039 is selected. The consequence of leaving it as-is is that Staff Office L1-048 has no VAV telemetry in the delivered graph. Restoring the 3 points is a one-line change if the client confirms.</t>
+          <t>RESOLVED. Client direction 2026-09-04, confirming this was an omission in the selection rather than a decision: the box is real in the asset register, it serves a room no other box serves, and the near-identical 039 is selected. Leaving it out would have left Staff Office L1-048 with no VAV telemetry in the delivered graph. The sheet now carries four unselected ids, all exempt by name and for stated reasons: ContributionFraction plus these three.</t>
         </is>
       </c>
       <c r="I44" s="19" t="inlineStr">
         <is>
-          <t>3 points dropped (restorable)</t>
+          <t>3 points restored, 6 rows</t>
         </is>
       </c>
     </row>

</xml_diff>